<commit_message>
Remove all Vietnamese metadata; standardize Excel and JSON descriptions to 100% English
</commit_message>
<xml_diff>
--- a/report/mearsuring-profile/MP-01_Hoist_Fast_Safety_Sync.xlsx
+++ b/report/mearsuring-profile/MP-01_Hoist_Fast_Safety_Sync.xlsx
@@ -633,9 +633,8 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>▶  MP-01 Hoist Fast - Safety &amp; Sync Critical (Giám Sát Đồng Bộ Tời Tốc Độ Cao &amp; An Toàn)  |  Tests: LOAD-002, LOAD-003, LOAD-006, LOAD-009, LOAD-012, LOAD-015, PERF-001
-Description (EN): High-speed monitoring of hoist winch positions, currents, temperatures, and synchronization to detect mechanical errors during heavy lift tests.
-Mô tả (VI): Giám sát tần suất cao (250ms) vị trí tời nâng, dòng điện, nhiệt độ và sai lệch đồng bộ cơ khí (AB, CD) để phát hiện lỗi cơ cấu nâng hạ và đảm bảo an toàn thử tải.</t>
+          <t>▶  MP-01 Hoist Fast - Safety &amp; Sync Critical  |  Tests: LOAD-002, LOAD-003, LOAD-006, LOAD-009, LOAD-012, LOAD-015, PERF-001
+Description: High-speed monitoring of hoist winch positions, currents, temperatures, and synchronization to detect mechanical errors during heavy lift tests.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: document telemetry FormatBinary pattern and update handoff
</commit_message>
<xml_diff>
--- a/report/mearsuring-profile/MP-01_Hoist_Fast_Safety_Sync.xlsx
+++ b/report/mearsuring-profile/MP-01_Hoist_Fast_Safety_Sync.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\local\opencode\codesys\report\measuring-profile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9669ECF0-E7BF-4BAE-A978-5407A04346D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51ADE571-5FF6-450E-B220-B64A4DA23C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="103">
   <si>
     <t>▶  MP-01 Hoist Fast - Safety &amp; Sync Critical  |  Tests: LOAD-002, LOAD-003, LOAD-006, LOAD-009, LOAD-012, LOAD-015, PERF-001
 Description: High-speed monitoring of hoist winch positions, currents, temperatures, and synchronization to detect mechanical errors during heavy lift tests.</t>
@@ -276,6 +276,60 @@
   </si>
   <si>
     <t>Reported hoist lift/lower cycle count</t>
+  </si>
+  <si>
+    <t>batt_voltage_winchB</t>
+  </si>
+  <si>
+    <t>Measured battery voltage of winch B</t>
+  </si>
+  <si>
+    <t>CANBusDrive/cWinchB/BattVoltage</t>
+  </si>
+  <si>
+    <t>batt_voltage_winchC</t>
+  </si>
+  <si>
+    <t>Measured battery voltage of winch C</t>
+  </si>
+  <si>
+    <t>CANBusDrive/cWinchC/BattVoltage</t>
+  </si>
+  <si>
+    <t>batt_voltage_winchD</t>
+  </si>
+  <si>
+    <t>Measured battery voltage of winch D</t>
+  </si>
+  <si>
+    <t>CANBusDrive/cWinchD/BattVoltage</t>
+  </si>
+  <si>
+    <t>torque_winchB</t>
+  </si>
+  <si>
+    <t>Estimated motor torque of winch B</t>
+  </si>
+  <si>
+    <t>CANBusDrive/cWinchB/Torque</t>
+  </si>
+  <si>
+    <t>torque_winchC</t>
+  </si>
+  <si>
+    <t>Estimated motor torque of winch C</t>
+  </si>
+  <si>
+    <t>CANBusDrive/cWinchC/Torque</t>
+  </si>
+  <si>
+    <t>torque_winchD</t>
+  </si>
+  <si>
+    <t>Estimated motor torque of winch D</t>
+  </si>
+  <si>
+    <t>CANBusDrive/cWinchD/Torque</t>
   </si>
 </sst>
 </file>
@@ -808,14 +862,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="42.7109375" customWidth="1"/>
     <col min="4" max="4" width="29.28515625" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="9" max="9" width="32" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1180,246 +1234,246 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="10">
-        <v>-3000</v>
-      </c>
-      <c r="F14" s="10">
-        <v>3000</v>
+      <c r="A14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>900</v>
       </c>
       <c r="G14" s="5">
         <v>10</v>
       </c>
-      <c r="H14" s="11">
-        <v>100</v>
-      </c>
-      <c r="I14" s="9" t="s">
+      <c r="H14" s="6">
+        <v>100</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>51</v>
+        <v>88</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="E15" s="4">
         <v>0</v>
       </c>
       <c r="F15" s="4">
-        <v>10</v>
-      </c>
-      <c r="G15" s="12">
-        <v>250</v>
+        <v>900</v>
+      </c>
+      <c r="G15" s="5">
+        <v>10</v>
       </c>
       <c r="H15" s="6">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E16" s="10">
+      <c r="A16" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="4">
         <v>0</v>
       </c>
-      <c r="F16" s="10">
-        <v>50000</v>
-      </c>
-      <c r="G16" s="12">
-        <v>250</v>
-      </c>
-      <c r="H16" s="11">
-        <v>4</v>
-      </c>
-      <c r="I16" s="9" t="s">
+      <c r="F16" s="4">
+        <v>900</v>
+      </c>
+      <c r="G16" s="5">
+        <v>10</v>
+      </c>
+      <c r="H16" s="6">
+        <v>100</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="4">
-        <v>-10</v>
-      </c>
-      <c r="F17" s="4">
-        <v>10</v>
+      <c r="A17" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="10">
+        <v>-3000</v>
+      </c>
+      <c r="F17" s="10">
+        <v>3000</v>
       </c>
       <c r="G17" s="5">
         <v>10</v>
       </c>
-      <c r="H17" s="6">
-        <v>100</v>
-      </c>
-      <c r="I17" s="7" t="s">
+      <c r="H17" s="11">
+        <v>100</v>
+      </c>
+      <c r="I17" s="9" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>62</v>
+        <v>95</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="E18" s="10">
-        <v>-20</v>
+        <v>-3000</v>
       </c>
       <c r="F18" s="10">
-        <v>200</v>
-      </c>
-      <c r="G18" s="13">
-        <v>1000</v>
+        <v>3000</v>
+      </c>
+      <c r="G18" s="5">
+        <v>10</v>
       </c>
       <c r="H18" s="11">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>65</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="4">
-        <v>-20</v>
-      </c>
-      <c r="F19" s="4">
-        <v>200</v>
-      </c>
-      <c r="G19" s="13">
-        <v>1000</v>
-      </c>
-      <c r="H19" s="6">
-        <v>1</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>65</v>
+      <c r="A19" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="10">
+        <v>-3000</v>
+      </c>
+      <c r="F19" s="10">
+        <v>3000</v>
+      </c>
+      <c r="G19" s="5">
+        <v>10</v>
+      </c>
+      <c r="H19" s="11">
+        <v>100</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="E20" s="10">
-        <v>-20</v>
+        <v>-3000</v>
       </c>
       <c r="F20" s="10">
-        <v>200</v>
-      </c>
-      <c r="G20" s="13">
-        <v>1000</v>
+        <v>3000</v>
+      </c>
+      <c r="G20" s="5">
+        <v>10</v>
       </c>
       <c r="H20" s="11">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>65</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E21" s="4">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="F21" s="4">
-        <v>200</v>
-      </c>
-      <c r="G21" s="13">
-        <v>1000</v>
+        <v>10</v>
+      </c>
+      <c r="G21" s="12">
+        <v>250</v>
       </c>
       <c r="H21" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>65</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>54</v>
@@ -1428,7 +1482,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="10">
-        <v>65535</v>
+        <v>50000</v>
       </c>
       <c r="G22" s="12">
         <v>250</v>
@@ -1442,80 +1496,80 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="E23" s="4">
-        <v>-800</v>
+        <v>-10</v>
       </c>
       <c r="F23" s="4">
-        <v>800</v>
-      </c>
-      <c r="G23" s="12">
-        <v>250</v>
+        <v>10</v>
+      </c>
+      <c r="G23" s="5">
+        <v>10</v>
       </c>
       <c r="H23" s="6">
-        <v>4</v>
-      </c>
-      <c r="I23" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E24" s="10">
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="F24" s="10">
+        <v>200</v>
+      </c>
+      <c r="G24" s="13">
         <v>1000</v>
       </c>
-      <c r="G24" s="12">
-        <v>250</v>
-      </c>
       <c r="H24" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="E25" s="4">
-        <v>0</v>
+        <v>-20</v>
       </c>
       <c r="F25" s="4">
-        <v>9999</v>
+        <v>200</v>
       </c>
       <c r="G25" s="13">
         <v>1000</v>
@@ -1524,6 +1578,180 @@
         <v>1</v>
       </c>
       <c r="I25" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="10">
+        <v>-20</v>
+      </c>
+      <c r="F26" s="10">
+        <v>200</v>
+      </c>
+      <c r="G26" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H26" s="11">
+        <v>1</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="4">
+        <v>-20</v>
+      </c>
+      <c r="F27" s="4">
+        <v>200</v>
+      </c>
+      <c r="G27" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H27" s="6">
+        <v>1</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" s="10">
+        <v>0</v>
+      </c>
+      <c r="F28" s="10">
+        <v>65535</v>
+      </c>
+      <c r="G28" s="12">
+        <v>250</v>
+      </c>
+      <c r="H28" s="11">
+        <v>4</v>
+      </c>
+      <c r="I28" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="4">
+        <v>-800</v>
+      </c>
+      <c r="F29" s="4">
+        <v>800</v>
+      </c>
+      <c r="G29" s="12">
+        <v>250</v>
+      </c>
+      <c r="H29" s="6">
+        <v>4</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30" s="10">
+        <v>0</v>
+      </c>
+      <c r="F30" s="10">
+        <v>1000</v>
+      </c>
+      <c r="G30" s="12">
+        <v>250</v>
+      </c>
+      <c r="H30" s="11">
+        <v>4</v>
+      </c>
+      <c r="I30" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31" s="4">
+        <v>0</v>
+      </c>
+      <c r="F31" s="4">
+        <v>9999</v>
+      </c>
+      <c r="G31" s="13">
+        <v>1000</v>
+      </c>
+      <c r="H31" s="6">
+        <v>1</v>
+      </c>
+      <c r="I31" s="3" t="s">
         <v>65</v>
       </c>
     </row>

</xml_diff>